<commit_message>
test: force an explainable demo trade-off
</commit_message>
<xml_diff>
--- a/data/demo-showcase/demo_showcase.xlsx
+++ b/data/demo-showcase/demo_showcase.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demo Summary" sheetId="1" r:id="Re4b8aeece2c74957"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Courses" sheetId="2" r:id="R04c11df552d4409e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Student Preferences" sheetId="3" r:id="R914fa10605ff46bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructor Preferences" sheetId="4" r:id="R028a343fdd464a3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hard Conflicts" sheetId="5" r:id="R07f8041fc9254c59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="Rce89e6025f4940a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demo Summary" sheetId="1" r:id="R1447742bf11e4af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Courses" sheetId="2" r:id="Rbfac7b40f25042a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Student Preferences" sheetId="3" r:id="R83388fad1d6d42fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructor Preferences" sheetId="4" r:id="R5b51a6e8bf78445c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hard Conflicts" sheetId="5" r:id="R50b7502b914c418f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="Re5400425cb8341e5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -466,7 +466,7 @@
         <x:v>Anonymous students</x:v>
       </x:c>
       <x:c r="B6" s="17" t="n">
-        <x:v>30</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C6" s="13"/>
       <x:c r="D6" s="18" t="str">
@@ -482,7 +482,7 @@
         <x:v>Preference rows</x:v>
       </x:c>
       <x:c r="B7" s="17" t="n">
-        <x:v>120</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="C7" s="13"/>
       <x:c r="D7" s="18" t="str">
@@ -502,7 +502,7 @@
       </x:c>
       <x:c r="C8" s="13"/>
       <x:c r="D8" s="18" t="str">
-        <x:v>Student demand forms four interpretable preference clusters.</x:v>
+        <x:v>Four demand clusters plus six coverage profiles connect every elective pair.</x:v>
       </x:c>
       <x:c r="E8" s="18" t="str"/>
       <x:c r="F8" s="18" t="str"/>
@@ -2374,13 +2374,277 @@
       </x:c>
     </x:row>
     <x:row r="121" ht="15" hidden="0" customHeight="1">
-      <x:c r="A121" s="26" t="str">
+      <x:c r="A121" s="25" t="str">
         <x:v>DEMO030</x:v>
       </x:c>
-      <x:c r="B121" s="26" t="str">
+      <x:c r="B121" s="25" t="str">
         <x:v>EE5141</x:v>
       </x:c>
-      <x:c r="C121" s="26" t="str">
+      <x:c r="C121" s="25" t="str">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="15" hidden="0" customHeight="1">
+      <x:c r="A122" s="25" t="str">
+        <x:v>DEMO031</x:v>
+      </x:c>
+      <x:c r="B122" s="25" t="str">
+        <x:v>EE6180</x:v>
+      </x:c>
+      <x:c r="C122" s="25" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="15" hidden="0" customHeight="1">
+      <x:c r="A123" s="25" t="str">
+        <x:v>DEMO031</x:v>
+      </x:c>
+      <x:c r="B123" s="25" t="str">
+        <x:v>EE5178</x:v>
+      </x:c>
+      <x:c r="C123" s="25" t="str">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="15" hidden="0" customHeight="1">
+      <x:c r="A124" s="25" t="str">
+        <x:v>DEMO031</x:v>
+      </x:c>
+      <x:c r="B124" s="25" t="str">
+        <x:v>EE5175</x:v>
+      </x:c>
+      <x:c r="C124" s="25" t="str">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="15" hidden="0" customHeight="1">
+      <x:c r="A125" s="25" t="str">
+        <x:v>DEMO031</x:v>
+      </x:c>
+      <x:c r="B125" s="25" t="str">
+        <x:v>EE5150</x:v>
+      </x:c>
+      <x:c r="C125" s="25" t="str">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="15" hidden="0" customHeight="1">
+      <x:c r="A126" s="25" t="str">
+        <x:v>DEMO032</x:v>
+      </x:c>
+      <x:c r="B126" s="25" t="str">
+        <x:v>EE6180</x:v>
+      </x:c>
+      <x:c r="C126" s="25" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="15" hidden="0" customHeight="1">
+      <x:c r="A127" s="25" t="str">
+        <x:v>DEMO032</x:v>
+      </x:c>
+      <x:c r="B127" s="25" t="str">
+        <x:v>EE5178</x:v>
+      </x:c>
+      <x:c r="C127" s="25" t="str">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="15" hidden="0" customHeight="1">
+      <x:c r="A128" s="25" t="str">
+        <x:v>DEMO032</x:v>
+      </x:c>
+      <x:c r="B128" s="25" t="str">
+        <x:v>EE5141</x:v>
+      </x:c>
+      <x:c r="C128" s="25" t="str">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="15" hidden="0" customHeight="1">
+      <x:c r="A129" s="25" t="str">
+        <x:v>DEMO032</x:v>
+      </x:c>
+      <x:c r="B129" s="25" t="str">
+        <x:v>EE5112</x:v>
+      </x:c>
+      <x:c r="C129" s="25" t="str">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="15" hidden="0" customHeight="1">
+      <x:c r="A130" s="25" t="str">
+        <x:v>DEMO033</x:v>
+      </x:c>
+      <x:c r="B130" s="25" t="str">
+        <x:v>EE6180</x:v>
+      </x:c>
+      <x:c r="C130" s="25" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="15" hidden="0" customHeight="1">
+      <x:c r="A131" s="25" t="str">
+        <x:v>DEMO033</x:v>
+      </x:c>
+      <x:c r="B131" s="25" t="str">
+        <x:v>EE5178</x:v>
+      </x:c>
+      <x:c r="C131" s="25" t="str">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="15" hidden="0" customHeight="1">
+      <x:c r="A132" s="25" t="str">
+        <x:v>DEMO033</x:v>
+      </x:c>
+      <x:c r="B132" s="25" t="str">
+        <x:v>EE3110</x:v>
+      </x:c>
+      <x:c r="C132" s="25" t="str">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="15" hidden="0" customHeight="1">
+      <x:c r="A133" s="25" t="str">
+        <x:v>DEMO033</x:v>
+      </x:c>
+      <x:c r="B133" s="25" t="str">
+        <x:v>EE5143</x:v>
+      </x:c>
+      <x:c r="C133" s="25" t="str">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="15" hidden="0" customHeight="1">
+      <x:c r="A134" s="25" t="str">
+        <x:v>DEMO034</x:v>
+      </x:c>
+      <x:c r="B134" s="25" t="str">
+        <x:v>EE5175</x:v>
+      </x:c>
+      <x:c r="C134" s="25" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="15" hidden="0" customHeight="1">
+      <x:c r="A135" s="25" t="str">
+        <x:v>DEMO034</x:v>
+      </x:c>
+      <x:c r="B135" s="25" t="str">
+        <x:v>EE5150</x:v>
+      </x:c>
+      <x:c r="C135" s="25" t="str">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="15" hidden="0" customHeight="1">
+      <x:c r="A136" s="25" t="str">
+        <x:v>DEMO034</x:v>
+      </x:c>
+      <x:c r="B136" s="25" t="str">
+        <x:v>EE5141</x:v>
+      </x:c>
+      <x:c r="C136" s="25" t="str">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="15" hidden="0" customHeight="1">
+      <x:c r="A137" s="25" t="str">
+        <x:v>DEMO034</x:v>
+      </x:c>
+      <x:c r="B137" s="25" t="str">
+        <x:v>EE5112</x:v>
+      </x:c>
+      <x:c r="C137" s="25" t="str">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="15" hidden="0" customHeight="1">
+      <x:c r="A138" s="25" t="str">
+        <x:v>DEMO035</x:v>
+      </x:c>
+      <x:c r="B138" s="25" t="str">
+        <x:v>EE5175</x:v>
+      </x:c>
+      <x:c r="C138" s="25" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" ht="15" hidden="0" customHeight="1">
+      <x:c r="A139" s="25" t="str">
+        <x:v>DEMO035</x:v>
+      </x:c>
+      <x:c r="B139" s="25" t="str">
+        <x:v>EE5150</x:v>
+      </x:c>
+      <x:c r="C139" s="25" t="str">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" ht="15" hidden="0" customHeight="1">
+      <x:c r="A140" s="25" t="str">
+        <x:v>DEMO035</x:v>
+      </x:c>
+      <x:c r="B140" s="25" t="str">
+        <x:v>EE3110</x:v>
+      </x:c>
+      <x:c r="C140" s="25" t="str">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="15" hidden="0" customHeight="1">
+      <x:c r="A141" s="25" t="str">
+        <x:v>DEMO035</x:v>
+      </x:c>
+      <x:c r="B141" s="25" t="str">
+        <x:v>EE5143</x:v>
+      </x:c>
+      <x:c r="C141" s="25" t="str">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="15" hidden="0" customHeight="1">
+      <x:c r="A142" s="25" t="str">
+        <x:v>DEMO036</x:v>
+      </x:c>
+      <x:c r="B142" s="25" t="str">
+        <x:v>EE5141</x:v>
+      </x:c>
+      <x:c r="C142" s="25" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" ht="15" hidden="0" customHeight="1">
+      <x:c r="A143" s="25" t="str">
+        <x:v>DEMO036</x:v>
+      </x:c>
+      <x:c r="B143" s="25" t="str">
+        <x:v>EE5112</x:v>
+      </x:c>
+      <x:c r="C143" s="25" t="str">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="15" hidden="0" customHeight="1">
+      <x:c r="A144" s="25" t="str">
+        <x:v>DEMO036</x:v>
+      </x:c>
+      <x:c r="B144" s="25" t="str">
+        <x:v>EE3110</x:v>
+      </x:c>
+      <x:c r="C144" s="25" t="str">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" ht="15" hidden="0" customHeight="1">
+      <x:c r="A145" s="26" t="str">
+        <x:v>DEMO036</x:v>
+      </x:c>
+      <x:c r="B145" s="26" t="str">
+        <x:v>EE5143</x:v>
+      </x:c>
+      <x:c r="C145" s="26" t="str">
         <x:v>4</x:v>
       </x:c>
     </x:row>

</xml_diff>